<commit_message>
Implemented dynamic acute benchmark names taken from dose response library
</commit_message>
<xml_diff>
--- a/resources/Dose_Response_Library.xlsx
+++ b/resources/Dose_Response_Library.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git_HEM4\HEM4\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A8EA491-702F-4ABF-A6CD-FFA881D04658}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{506C743B-508F-4D36-9B38-AF7495FC9485}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1959,11 +1959,11 @@
     <t>106-94-5</t>
   </si>
   <si>
-    <t>Acute NCREL
+    <t>ERPG-2
 (mg/m3)</t>
   </si>
   <si>
-    <t>NCERPG-2
+    <t>Acute REL
 (mg/m3)</t>
   </si>
 </sst>
@@ -3010,10 +3010,10 @@
         <v>6</v>
       </c>
       <c r="I1" s="3" t="s">
+        <v>629</v>
+      </c>
+      <c r="J1" s="3" t="s">
         <v>630</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>629</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">

</xml_diff>